<commit_message>
Cleaned scripts and updated summaries and plots
</commit_message>
<xml_diff>
--- a/builds/systematic_review/sys_rev_filt.xlsx
+++ b/builds/systematic_review/sys_rev_filt.xlsx
@@ -8,15 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://connectqutedu-my.sharepoint.com/personal/n11878916_qut_edu_au/Documents/Documents/Sixth mass extinction/Luna_project/rat_evidence_review/builds/systematic_review/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_8602AB03BDA89AEF9A745B61E3BFCA26DBC0C691" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9432C430-5943-430C-A189-E4A304468ECE}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_8602AB03BDA89AEF9A745B61E3BFCA26DBC0C691" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F81F917-DC13-457D-ACF6-4084CE731731}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sys_rev_all_included" sheetId="1" r:id="rId1"/>
     <sheet name="sys_rev_all_extant" sheetId="2" r:id="rId2"/>
     <sheet name="sys_rev_all_extant_multi-island" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">sys_rev_all_extant!$A$1:$D$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'sys_rev_all_extant_multi-island'!$A$1:$D$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sys_rev_all_included!$A$1:$D$33</definedName>
+  </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
@@ -133,6 +138,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -422,6 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -487,7 +497,7 @@
         <v>2.3668639053254439</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -515,7 +525,7 @@
         <v>14.79289940828402</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -529,7 +539,7 @@
         <v>1.775147928994083</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -543,7 +553,7 @@
         <v>3.550295857988166</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -557,7 +567,7 @@
         <v>45.454545454545453</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -571,7 +581,7 @@
         <v>45.454545454545453</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -585,7 +595,7 @@
         <v>3.0303030303030298</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -599,7 +609,7 @@
         <v>6.0606060606060614</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -613,7 +623,7 @@
         <v>8.6206896551724146</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -627,7 +637,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -641,7 +651,7 @@
         <v>8.6206896551724146</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -655,7 +665,7 @@
         <v>2.5862068965517242</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -669,7 +679,7 @@
         <v>0.86206896551724133</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -683,7 +693,7 @@
         <v>1.7241379310344831</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -697,7 +707,7 @@
         <v>2.5862068965517242</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -711,7 +721,7 @@
         <v>74.157303370786522</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -725,7 +735,7 @@
         <v>7.3033707865168536</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -739,7 +749,7 @@
         <v>12.921348314606741</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -753,7 +763,7 @@
         <v>2.808988764044944</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -767,7 +777,7 @@
         <v>0.5617977528089888</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>11</v>
       </c>
@@ -781,7 +791,7 @@
         <v>0.5617977528089888</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>7</v>
       </c>
@@ -795,7 +805,7 @@
         <v>1.685393258426966</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -809,7 +819,7 @@
         <v>62.989323843416358</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>6</v>
       </c>
@@ -823,7 +833,7 @@
         <v>11.032028469750889</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>7</v>
       </c>
@@ -837,7 +847,7 @@
         <v>2.8469750889679708</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -851,7 +861,7 @@
         <v>6.4056939501779357</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>9</v>
       </c>
@@ -865,7 +875,7 @@
         <v>12.09964412811388</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>10</v>
       </c>
@@ -879,7 +889,7 @@
         <v>1.4234875444839861</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -894,12 +904,28 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D33" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="All studies are not in support"/>
+        <filter val="Lethal program in support"/>
+        <filter val="No studies found"/>
+        <filter val="Only predation in support"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="All rodents"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -979,7 +1005,7 @@
         <v>17.6056338028169</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -993,7 +1019,7 @@
         <v>4.5774647887323949</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1007,7 +1033,7 @@
         <v>2.112676056338028</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1021,7 +1047,7 @@
         <v>4.225352112676056</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1035,7 +1061,7 @@
         <v>45.454545454545453</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1049,7 +1075,7 @@
         <v>45.454545454545453</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1063,7 +1089,7 @@
         <v>3.0303030303030298</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1077,7 +1103,7 @@
         <v>6.0606060606060614</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1091,7 +1117,7 @@
         <v>10.22727272727273</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1105,7 +1131,7 @@
         <v>70.454545454545453</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1119,7 +1145,7 @@
         <v>11.36363636363636</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1133,7 +1159,7 @@
         <v>1.136363636363636</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -1147,7 +1173,7 @@
         <v>1.136363636363636</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -1161,7 +1187,7 @@
         <v>2.2727272727272729</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -1175,7 +1201,7 @@
         <v>3.4090909090909092</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -1189,7 +1215,7 @@
         <v>69.594594594594597</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -1203,7 +1229,7 @@
         <v>8.7837837837837842</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -1217,7 +1243,7 @@
         <v>15.54054054054054</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -1231,7 +1257,7 @@
         <v>2.7027027027027031</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>14</v>
       </c>
@@ -1245,7 +1271,7 @@
         <v>0.67567567567567566</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>14</v>
       </c>
@@ -1259,7 +1285,7 @@
         <v>0.67567567567567566</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>14</v>
       </c>
@@ -1273,7 +1299,7 @@
         <v>2.0270270270270272</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -1287,7 +1313,7 @@
         <v>59.82905982905983</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>15</v>
       </c>
@@ -1301,7 +1327,7 @@
         <v>12.39316239316239</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>15</v>
       </c>
@@ -1315,7 +1341,7 @@
         <v>3.4188034188034191</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>15</v>
       </c>
@@ -1329,7 +1355,7 @@
         <v>14.52991452991453</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>15</v>
       </c>
@@ -1343,7 +1369,7 @@
         <v>4.2735042735042734</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -1357,7 +1383,7 @@
         <v>1.70940170940171</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>15</v>
       </c>
@@ -1372,12 +1398,28 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D33" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="All rodents"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="All studies are not in support"/>
+        <filter val="Lethal program in support"/>
+        <filter val="No studies found"/>
+        <filter val="Only predation in support"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1457,7 +1499,7 @@
         <v>19.125683060109289</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1471,7 +1513,7 @@
         <v>6.0109289617486326</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1485,7 +1527,7 @@
         <v>2.1857923497267762</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -1499,7 +1541,7 @@
         <v>6.557377049180328</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1513,7 +1555,7 @@
         <v>40.74074074074074</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1527,7 +1569,7 @@
         <v>48.148148148148152</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1541,7 +1583,7 @@
         <v>3.7037037037037028</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1555,7 +1597,7 @@
         <v>7.4074074074074074</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1569,7 +1611,7 @@
         <v>65.454545454545453</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1583,7 +1625,7 @@
         <v>10.90909090909091</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1597,7 +1639,7 @@
         <v>12.72727272727273</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1611,7 +1653,7 @@
         <v>1.8181818181818179</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -1625,7 +1667,7 @@
         <v>1.8181818181818179</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -1639,7 +1681,7 @@
         <v>3.6363636363636358</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -1653,7 +1695,7 @@
         <v>3.6363636363636358</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -1667,7 +1709,7 @@
         <v>66.34615384615384</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -1681,7 +1723,7 @@
         <v>10.57692307692308</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -1695,7 +1737,7 @@
         <v>15.38461538461539</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -1709,7 +1751,7 @@
         <v>3.8461538461538458</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>14</v>
       </c>
@@ -1723,7 +1765,7 @@
         <v>0.96153846153846156</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>14</v>
       </c>
@@ -1737,7 +1779,7 @@
         <v>0.96153846153846156</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>14</v>
       </c>
@@ -1751,7 +1793,7 @@
         <v>1.9230769230769229</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -1765,7 +1807,7 @@
         <v>53.146853146853147</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>15</v>
       </c>
@@ -1779,7 +1821,7 @@
         <v>2.7972027972027971</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>15</v>
       </c>
@@ -1793,7 +1835,7 @@
         <v>16.08391608391608</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>15</v>
       </c>
@@ -1807,7 +1849,7 @@
         <v>14.68531468531468</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>15</v>
       </c>
@@ -1821,7 +1863,7 @@
         <v>5.5944055944055942</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -1835,7 +1877,7 @@
         <v>1.398601398601399</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>15</v>
       </c>
@@ -1850,6 +1892,21 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D33" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="All rodents"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="All studies are not in support"/>
+        <filter val="Lethal program in support"/>
+        <filter val="No studies found"/>
+        <filter val="Only predation in support"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>